<commit_message>
Bases limited to 1 when a MV is present
</commit_message>
<xml_diff>
--- a/data/Inputs.xlsx
+++ b/data/Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d3dd903d477a9e4d/02_ME/ME54015/OWF_Vessel-Fleet-Optimization/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{4E655DA3-6644-44D5-B8A3-390376DF86AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B52679FC-B784-4589-B590-BD14CDDAF4C5}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{4E655DA3-6644-44D5-B8A3-390376DF86AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C650A8AB-C103-4C56-8487-AEA7D9908CDF}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="8" activeTab="12" xr2:uid="{5CDB4E5C-34BF-4466-8F20-CB91BE55E2BE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="8" activeTab="8" xr2:uid="{5CDB4E5C-34BF-4466-8F20-CB91BE55E2BE}"/>
   </bookViews>
   <sheets>
     <sheet name="general" sheetId="5" r:id="rId1"/>
@@ -730,10 +730,10 @@
         <v>S1</v>
       </c>
       <c r="B2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -747,7 +747,7 @@
         <v>0</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -781,13 +781,13 @@
         <v>S1</v>
       </c>
       <c r="B2">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="C2">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="D2">
-        <v>15</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -795,13 +795,13 @@
         <v>S2</v>
       </c>
       <c r="B3">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="C3">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="D3">
-        <v>10</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
initial result - compare
</commit_message>
<xml_diff>
--- a/data/Inputs.xlsx
+++ b/data/Inputs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d3dd903d477a9e4d/02_ME/ME54015/OWF_Vessel-Fleet-Optimization/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="13_ncr:1_{4E655DA3-6644-44D5-B8A3-390376DF86AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1267FFAC-C233-460D-9ACB-7991AC09EBCA}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="13_ncr:1_{4E655DA3-6644-44D5-B8A3-390376DF86AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1AF75254-8B48-4E78-B32B-6AD841145544}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="8" activeTab="11" xr2:uid="{5CDB4E5C-34BF-4466-8F20-CB91BE55E2BE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="8" activeTab="10" xr2:uid="{5CDB4E5C-34BF-4466-8F20-CB91BE55E2BE}"/>
   </bookViews>
   <sheets>
     <sheet name="general" sheetId="5" r:id="rId1"/>
@@ -733,7 +733,7 @@
         <v>3</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -747,7 +747,7 @@
         <v>0</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -787,7 +787,7 @@
         <v>100</v>
       </c>
       <c r="D2">
-        <v>40</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -801,7 +801,7 @@
         <v>100</v>
       </c>
       <c r="D3">
-        <v>100</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>